<commit_message>
Removed python iles moved the hardcoded references to the configuration file
</commit_message>
<xml_diff>
--- a/SourceFiles/ProspectData.xlsx
+++ b/SourceFiles/ProspectData.xlsx
@@ -126,7 +126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -325,7 +325,36 @@
       <c r="G7" s="0" t="b">
         <v>0</v>
       </c>
+      <c r="H7" s="0" t="s">
+        <v>10</v>
+      </c>
       <c r="I7" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" s="0">
         <v>0</v>
       </c>
     </row>

</xml_diff>